<commit_message>
v2: fixes 13-18, fecha_remate revertido, docs actualizados
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/causas_ojv_template.xlsx
+++ b/causas_ojv_template.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B234"/>
+  <dimension ref="A1:B235"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3339,6 +3339,18 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>C.A. de Santiago</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Juzgado de Letras de Colina</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>